<commit_message>
Apply working tree updates and builder validation/export flow changes
</commit_message>
<xml_diff>
--- a/data/IMPORTED DATA/MASTER/sun_simulator_data.xlsx
+++ b/data/IMPORTED DATA/MASTER/sun_simulator_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,11 +461,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RW001</t>
+          <t>E2E001</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C2" t="n">
         <v>10</v>
@@ -477,11 +477,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RW002</t>
+          <t>E2E002</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>
@@ -493,11 +493,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RW003</t>
+          <t>E2E003</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="C4" t="n">
         <v>10</v>
@@ -509,7 +509,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RW004</t>
+          <t>E2E004</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -519,38 +519,6 @@
         <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>RW005</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>225</v>
-      </c>
-      <c r="C6" t="n">
-        <v>11</v>
-      </c>
-      <c r="D6" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>RW006</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>230</v>
-      </c>
-      <c r="C7" t="n">
-        <v>11</v>
-      </c>
-      <c r="D7" t="n">
         <v>42</v>
       </c>
     </row>

</xml_diff>